<commit_message>
CoC analysis and hu supply updates
Added rate per 10k pop to CoC analysis, refined hu supply
</commit_message>
<xml_diff>
--- a/2026_update/exploratory_work/coc_exploration_export.xlsx
+++ b/2026_update/exploratory_work/coc_exploration_export.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="112">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="115">
   <si>
     <t xml:space="preserve">coc_num</t>
   </si>
@@ -348,7 +348,16 @@
     <t xml:space="preserve">Boston CoC</t>
   </si>
   <si>
-    <t xml:space="preserve">PSRC Region – King, Pierce, Snohomish</t>
+    <t xml:space="preserve">total_per_10k</t>
+  </si>
+  <si>
+    <t xml:space="preserve">unsheltered_per_10k</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sheltered_per_10k</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3Cnty – King, Pierce, Snohomish</t>
   </si>
 </sst>
 </file>
@@ -2507,13 +2516,20 @@
       <c r="K1" t="s">
         <v>10</v>
       </c>
+      <c r="L1" t="s">
+        <v>111</v>
+      </c>
+      <c r="M1" t="s">
+        <v>112</v>
+      </c>
+      <c r="N1" t="s">
+        <v>113</v>
+      </c>
     </row>
     <row r="2">
-      <c r="A2" t="s">
-        <v>29</v>
-      </c>
+      <c r="A2"/>
       <c r="B2" t="s">
-        <v>30</v>
+        <v>114</v>
       </c>
       <c r="C2" t="n">
         <v>2015</v>
@@ -2522,31 +2538,42 @@
         <v>2024</v>
       </c>
       <c r="E2" t="n">
-        <v>16868</v>
+        <v>20690</v>
       </c>
       <c r="F2" t="n">
-        <v>7058</v>
+        <v>9039</v>
       </c>
       <c r="G2" t="n">
-        <v>9810</v>
+        <v>11651</v>
       </c>
       <c r="H2" t="n">
-        <v>0.666469077257459</v>
+        <v>0.691188491090404</v>
       </c>
       <c r="I2" t="n">
-        <v>0.116948884317139</v>
+        <v>0.16212393931602</v>
       </c>
       <c r="J2" t="n">
-        <v>1.57954246647384</v>
+        <v>1.61467684021544</v>
       </c>
       <c r="K2" t="n">
-        <v>0.581574579084657</v>
+        <v>0.563122281295312</v>
+      </c>
+      <c r="L2" t="n">
+        <v>49.3</v>
+      </c>
+      <c r="M2" t="n">
+        <v>27.8</v>
+      </c>
+      <c r="N2" t="n">
+        <v>21.5</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3"/>
+      <c r="A3" t="s">
+        <v>35</v>
+      </c>
       <c r="B3" t="s">
-        <v>111</v>
+        <v>36</v>
       </c>
       <c r="C3" t="n">
         <v>2015</v>
@@ -2555,33 +2582,42 @@
         <v>2024</v>
       </c>
       <c r="E3" t="n">
-        <v>20690</v>
+        <v>1161</v>
       </c>
       <c r="F3" t="n">
-        <v>9039</v>
+        <v>536</v>
       </c>
       <c r="G3" t="n">
-        <v>11651</v>
+        <v>625</v>
       </c>
       <c r="H3" t="n">
-        <v>0.691188491090404</v>
+        <v>0.400482509047045</v>
       </c>
       <c r="I3" t="n">
-        <v>0.16212393931602</v>
+        <v>0.0367504835589942</v>
       </c>
       <c r="J3" t="n">
-        <v>1.61467684021544</v>
+        <v>1.00320512820513</v>
       </c>
       <c r="K3" t="n">
-        <v>0.563122281295312</v>
+        <v>0.53832902670112</v>
+      </c>
+      <c r="L3" t="n">
+        <v>13.4</v>
+      </c>
+      <c r="M3" t="n">
+        <v>7.2</v>
+      </c>
+      <c r="N3" t="n">
+        <v>6.2</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="B4" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="C4" t="n">
         <v>2015</v>
@@ -2590,25 +2626,34 @@
         <v>2024</v>
       </c>
       <c r="E4" t="n">
-        <v>1161</v>
+        <v>16868</v>
       </c>
       <c r="F4" t="n">
-        <v>536</v>
+        <v>7058</v>
       </c>
       <c r="G4" t="n">
-        <v>625</v>
+        <v>9810</v>
       </c>
       <c r="H4" t="n">
-        <v>0.400482509047045</v>
+        <v>0.666469077257459</v>
       </c>
       <c r="I4" t="n">
-        <v>0.0367504835589942</v>
+        <v>0.116948884317139</v>
       </c>
       <c r="J4" t="n">
-        <v>1.00320512820513</v>
+        <v>1.57954246647384</v>
       </c>
       <c r="K4" t="n">
-        <v>0.53832902670112</v>
+        <v>0.581574579084657</v>
+      </c>
+      <c r="L4" t="n">
+        <v>70.9</v>
+      </c>
+      <c r="M4" t="n">
+        <v>41.3</v>
+      </c>
+      <c r="N4" t="n">
+        <v>29.7</v>
       </c>
     </row>
     <row r="5">
@@ -2644,6 +2689,15 @@
       </c>
       <c r="K5" t="n">
         <v>0.456971063509959</v>
+      </c>
+      <c r="L5" t="n">
+        <v>27.9</v>
+      </c>
+      <c r="M5" t="n">
+        <v>12.8</v>
+      </c>
+      <c r="N5" t="n">
+        <v>15.2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>